<commit_message>
Scripts for Orbitrap publication
</commit_message>
<xml_diff>
--- a/references_sulphate.xlsx
+++ b/references_sulphate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacksaville/Documents/Lab/Orbitrap/Data treatment/DC-2011-HSO4-sep2B-newstds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E5BB7E8-B9FF-154A-8860-2363D30396D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0B719B-114C-F542-88F3-EE74B93C4611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-47940" yWindow="-2600" windowWidth="22680" windowHeight="16300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="10660" windowHeight="16300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -578,9 +578,7 @@
         <v>0.22</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="2">
-        <v>0.36</v>
-      </c>
+      <c r="I2" s="2"/>
       <c r="J2" s="2">
         <v>-0.14399999999999999</v>
       </c>
@@ -631,9 +629,7 @@
         <v>0.26</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2">
-        <v>0.23</v>
-      </c>
+      <c r="I3" s="2"/>
       <c r="J3" s="2">
         <v>-0.32900000000000001</v>
       </c>

</xml_diff>